<commit_message>
feat: lock the 7-day kit to owning a car
Rewrite the deck, journal, and tracker around one desire: kendi arabam. Adds a ready 369 line, a driving SATS scene, and daily real-world car steps (budget, listings, insurance, deposit).

Co-authored-by: iremalisan <iremalisan@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/rehber/Yedi_Gunluk_Manifest_Takip.xlsx
+++ b/rehber/Yedi_Gunluk_Manifest_Takip.xlsx
@@ -11,7 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cümle" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WOOP" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Takip" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kaynaklar" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Araba" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kaynaklar" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Nasıl kullanılır'!$1:$5</definedName>
@@ -258,7 +259,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -332,6 +333,19 @@
     <xf numFmtId="0" fontId="12" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -882,14 +896,14 @@
     <row r="2" ht="28" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>7 günde hızlı manifest — takip tablosu</t>
+          <t>Kendi arabam — 7 günlük manifest takibi</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Sarı hücrelere yaz. Diğer sütunlar otomatik dolar. 7 gün aynı istek, aynı cümle.</t>
+          <t>Sarı hücrelere yaz. 7 günün tek isteği: kendi arabam. Aynı cümle, her gün 1 araba adımı.</t>
         </is>
       </c>
     </row>
@@ -918,7 +932,7 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Cümle sayfasına 369 cümleni yaz. Süzgeç 5/5 olana kadar küçült veya somutlaştır.</t>
+          <t>Cümle sayfasındaki araba cümlesini kilitle. Süzgeç 5/5 olsun.</t>
         </is>
       </c>
       <c r="D6" s="8" t="n"/>
@@ -934,7 +948,7 @@
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>WOOP sayfasında iç engeli ve eğer-o zaman planını doldur.</t>
+          <t>WOOP’ta ‘param yetmez’ engelini ve 2 dakikalık planı yaz.</t>
         </is>
       </c>
       <c r="D7" s="8" t="n"/>
@@ -950,7 +964,7 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Her gün Takip sayfasında Evet/Hayır işaretle, somut adımı bir cümleyle yaz, his notunu 1–10 ver.</t>
+          <t>Araba sayfasında bütçe, 2. el/yeni ve 3 modeli doldur.</t>
         </is>
       </c>
       <c r="D8" s="8" t="n"/>
@@ -966,7 +980,7 @@
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>Skor %80 altındaysa teknik ekleme; eksik katmanı (yazış / SATS / adım) tamamla.</t>
+          <t>Her gün Takip’te 369 + SATS + 1 araba adımını işaretle.</t>
         </is>
       </c>
       <c r="D9" s="8" t="n"/>
@@ -982,7 +996,7 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>7. gün özet satırını oku. Cümleyi gerekirse %10 netleştir, 21 güne uzat.</t>
+          <t>7. gün 3 adayı 1–2’ye indir; 21 güne bakış + biriktirme kilidi.</t>
         </is>
       </c>
       <c r="D10" s="8" t="n"/>
@@ -993,7 +1007,7 @@
     <row r="12" ht="28" customHeight="1">
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>Hız formülü: tek istek + 369 (3-6-9) + gece SATS + her gün 1 somut adım (WOOP).</t>
+          <t>Hız formülü: kendi arabam + 369 + gece direksiyon SATS + her gün 1 araba adımı.</t>
         </is>
       </c>
     </row>
@@ -1045,7 +1059,7 @@
     <row r="2">
       <c r="B2" s="12" t="inlineStr">
         <is>
-          <t>369 cümlesi</t>
+          <t>369 — kendi arabam</t>
         </is>
       </c>
     </row>
@@ -1066,7 +1080,7 @@
     <row r="6" ht="48" customHeight="1">
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>Bu ay nakit akışım rahatlasın</t>
+          <t>Kendi arabam</t>
         </is>
       </c>
       <c r="C6" s="15" t="n"/>
@@ -1084,7 +1098,7 @@
     <row r="8" ht="48" customHeight="1">
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>Çok minnettarım, bu ay faturalarım rahat ödeniyor ve kendimi güvende hissediyorum.</t>
+          <t>Çok minnettarım, kendi arabamla yola çıkıyorum ve özgür hissediyorum.</t>
         </is>
       </c>
       <c r="C8" s="15" t="n"/>
@@ -1102,7 +1116,7 @@
     <row r="10" ht="48" customHeight="1">
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>Mutfakta kahvemi içerken bakiyeyi görüp omuzlarımın düştüğünü hissediyorum.</t>
+          <t>Evin önünde kendi arabam park. Anahtarı çeviriyorum, kemer klik, geldik.</t>
         </is>
       </c>
       <c r="C10" s="15" t="n"/>
@@ -1120,7 +1134,7 @@
     <row r="12" ht="48" customHeight="1">
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>Bugün bir teklif maili gönderiyorum.</t>
+          <t>Bugün bütçe alt–üst ve 3 model adayını yazıyorum.</t>
         </is>
       </c>
       <c r="C12" s="15" t="n"/>
@@ -1151,7 +1165,7 @@
     <row r="15" ht="28" customHeight="1">
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>90 gün içinde mümkün mü?</t>
+          <t>90 günde peşinat / kredi / 2. el mümkün mü?</t>
         </is>
       </c>
       <c r="C15" s="16" t="inlineStr">
@@ -1166,7 +1180,7 @@
     <row r="16" ht="28" customHeight="1">
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>Hayal edince vücutta yumuşama var mı?</t>
+          <t>Direksiyonda hayal edince vücut yumuşuyor mu?</t>
         </is>
       </c>
       <c r="C16" s="16" t="inlineStr">
@@ -1181,7 +1195,7 @@
     <row r="17" ht="28" customHeight="1">
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>Atabileceğin en az bir adım var mı?</t>
+          <t>Bugün 1 araba adımı atabiliyor musun?</t>
         </is>
       </c>
       <c r="C17" s="16" t="inlineStr">
@@ -1196,7 +1210,7 @@
     <row r="18" ht="28" customHeight="1">
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>Başkasının iradesini zorlamıyor mu?</t>
+          <t>Başkasının sana almasını dayatmıyor musun?</t>
         </is>
       </c>
       <c r="C18" s="16" t="inlineStr">
@@ -1211,7 +1225,7 @@
     <row r="19" ht="28" customHeight="1">
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>Ölçülebilir mi? (tarih, tutar, olay)</t>
+          <t>Ölçülebilir mi? (bütçe aralığı, 2. el / yeni)</t>
         </is>
       </c>
       <c r="C19" s="16" t="inlineStr">
@@ -1337,7 +1351,7 @@
     <row r="11" ht="22" customHeight="1">
       <c r="B11" s="21" t="inlineStr">
         <is>
-          <t>Faturalar ödenmiş, omuzlar düşük, nefes rahat; ‘artık böyle’ hissi.</t>
+          <t>Kapıyı açıp koltuğa oturuyorum, kemer klik, ‘geldik’; omuzlar düşük.</t>
         </is>
       </c>
       <c r="C11" s="15" t="n"/>
@@ -1374,7 +1388,7 @@
     <row r="16" ht="22" customHeight="1">
       <c r="B16" s="21" t="inlineStr">
         <is>
-          <t>Öğleden sonra ‘nasıl olsa olmaz’ deyip telefonu kaydırmak.</t>
+          <t>Öğleden sonra ‘nasıl olsa araba alamam’ deyip ilan kaydırmak.</t>
         </is>
       </c>
       <c r="C16" s="15" t="n"/>
@@ -1411,7 +1425,7 @@
     <row r="21" ht="22" customHeight="1">
       <c r="B21" s="21" t="inlineStr">
         <is>
-          <t>Eğer kaydırmaya başlarsam, telefonu başka odaya koyar 2 dakikalık maili hemen bitiririm.</t>
+          <t>Eğer ‘alamam’ dersem, telefonu bırakır 1 satıcıya mesaj atar veya küçük transferi yaparım.</t>
         </is>
       </c>
       <c r="C21" s="15" t="n"/>
@@ -1434,7 +1448,7 @@
     <row r="25">
       <c r="B25" s="24" t="inlineStr">
         <is>
-          <t>Hazır iskelet: Eğer öğleden sonra “nasıl olsa olmaz” diye kaydırırsam, o zaman telefonu başka odaya koyar 2 dakikalık adımı hemen bitiririm.</t>
+          <t>Eğer öğleden sonra “nasıl olsa araba alamam” diye kaydırırsam, o zaman telefonu bırakır, bütçe satırını doldurur veya 1 satıcıya mesaj atarım.</t>
         </is>
       </c>
     </row>
@@ -1488,7 +1502,7 @@
     <row r="2">
       <c r="B2" s="12" t="inlineStr">
         <is>
-          <t>7 günlük ritim — sarı hücreleri doldur</t>
+          <t>7 günlük araba ritmi — sarı hücreleri doldur</t>
         </is>
       </c>
     </row>
@@ -1536,7 +1550,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Somut adım (ne yaptım?)</t>
+          <t>Somut araba adımı (ne yaptım?)</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -1596,7 +1610,7 @@
       </c>
       <c r="H6" s="16" t="inlineStr">
         <is>
-          <t>Teklif maili taslağını bitirdim.</t>
+          <t>Bütçe aralığını ve 3 model adayını yazdım.</t>
         </is>
       </c>
       <c r="I6" s="27" t="inlineStr">
@@ -1613,7 +1627,7 @@
       </c>
       <c r="L6" s="16" t="inlineStr">
         <is>
-          <t>Şüphe geldi, yazıp kapattım.</t>
+          <t>Şüphe geldi, yazıp kapattım. Anahtar sahnesine döndüm.</t>
         </is>
       </c>
     </row>
@@ -1866,11 +1880,391 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00C45476"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:F26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="12" t="inlineStr">
+        <is>
+          <t>Kendi arabam — gerçek dünya alanları</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Sarıya yaz. 3 modelden fazlası yok. Her gün Takip’teki adım buradan seçilir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr"/>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Alan</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Senin cevabın</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>İpucu</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6" ht="32" customHeight="1">
+      <c r="B6" s="35" t="inlineStr">
+        <is>
+          <t>Yeni / 2. el</t>
+        </is>
+      </c>
+      <c r="C6" s="36" t="inlineStr">
+        <is>
+          <t>2. el</t>
+        </is>
+      </c>
+      <c r="D6" s="17" t="n"/>
+      <c r="E6" s="37" t="inlineStr">
+        <is>
+          <t>İnanç eşiği zorlanıyorsa 2. el ile başla.</t>
+        </is>
+      </c>
+      <c r="F6" s="17" t="n"/>
+    </row>
+    <row r="7" ht="32" customHeight="1">
+      <c r="B7" s="35" t="inlineStr">
+        <is>
+          <t>Bütçe alt (TL)</t>
+        </is>
+      </c>
+      <c r="C7" s="36" t="inlineStr"/>
+      <c r="D7" s="17" t="n"/>
+      <c r="E7" s="37" t="inlineStr">
+        <is>
+          <t>Rahat verebileceğin taban. Sıfır yazma.</t>
+        </is>
+      </c>
+      <c r="F7" s="17" t="n"/>
+    </row>
+    <row r="8" ht="32" customHeight="1">
+      <c r="B8" s="35" t="inlineStr">
+        <is>
+          <t>Bütçe üst (TL)</t>
+        </is>
+      </c>
+      <c r="C8" s="36" t="inlineStr"/>
+      <c r="D8" s="17" t="n"/>
+      <c r="E8" s="37" t="inlineStr">
+        <is>
+          <t>Zorlama tavan. Üstünü 7 gün hayal etme.</t>
+        </is>
+      </c>
+      <c r="F8" s="17" t="n"/>
+    </row>
+    <row r="9" ht="32" customHeight="1">
+      <c r="B9" s="35" t="inlineStr">
+        <is>
+          <t>Peşinat hedefi (TL)</t>
+        </is>
+      </c>
+      <c r="C9" s="36" t="inlineStr"/>
+      <c r="D9" s="17" t="n"/>
+      <c r="E9" s="37" t="inlineStr">
+        <is>
+          <t>Bu hafta ayırabileceğin ilk tutar bile sayılır.</t>
+        </is>
+      </c>
+      <c r="F9" s="17" t="n"/>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="B10" s="35" t="inlineStr">
+        <is>
+          <t>Aylık biriktirme (TL)</t>
+        </is>
+      </c>
+      <c r="C10" s="36" t="inlineStr"/>
+      <c r="D10" s="17" t="n"/>
+      <c r="E10" s="37" t="inlineStr">
+        <is>
+          <t>Küçük ve tekrarlanabilir olsun.</t>
+        </is>
+      </c>
+      <c r="F10" s="17" t="n"/>
+    </row>
+    <row r="11" ht="32" customHeight="1">
+      <c r="B11" s="35" t="inlineStr">
+        <is>
+          <t>Ehliyet</t>
+        </is>
+      </c>
+      <c r="C11" s="36" t="inlineStr">
+        <is>
+          <t>Var / Yok / Yenileme</t>
+        </is>
+      </c>
+      <c r="D11" s="17" t="n"/>
+      <c r="E11" s="37" t="inlineStr">
+        <is>
+          <t>Yoksa SATS durmaz; ehliyet adımı da 7 güne girer.</t>
+        </is>
+      </c>
+      <c r="F11" s="17" t="n"/>
+    </row>
+    <row r="12" ht="32" customHeight="1">
+      <c r="B12" s="35" t="inlineStr">
+        <is>
+          <t>Aday 1</t>
+        </is>
+      </c>
+      <c r="C12" s="36" t="inlineStr"/>
+      <c r="D12" s="17" t="n"/>
+      <c r="E12" s="37" t="inlineStr">
+        <is>
+          <t>Tek cümle: marka + vites + yakıt.</t>
+        </is>
+      </c>
+      <c r="F12" s="17" t="n"/>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="B13" s="35" t="inlineStr">
+        <is>
+          <t>Aday 2</t>
+        </is>
+      </c>
+      <c r="C13" s="36" t="inlineStr"/>
+      <c r="D13" s="17" t="n"/>
+      <c r="E13" s="37" t="inlineStr"/>
+      <c r="F13" s="17" t="n"/>
+    </row>
+    <row r="14" ht="32" customHeight="1">
+      <c r="B14" s="35" t="inlineStr">
+        <is>
+          <t>Aday 3</t>
+        </is>
+      </c>
+      <c r="C14" s="36" t="inlineStr"/>
+      <c r="D14" s="17" t="n"/>
+      <c r="E14" s="37" t="inlineStr">
+        <is>
+          <t>4. aday yok. Beğenirsen birini çıkar.</t>
+        </is>
+      </c>
+      <c r="F14" s="17" t="n"/>
+    </row>
+    <row r="15" ht="32" customHeight="1">
+      <c r="B15" s="35" t="inlineStr">
+        <is>
+          <t>Trafik + kasko kaba (aylık)</t>
+        </is>
+      </c>
+      <c r="C15" s="36" t="inlineStr"/>
+      <c r="D15" s="17" t="n"/>
+      <c r="E15" s="37" t="inlineStr">
+        <is>
+          <t>Araba fiyatının yanında aylık gerçek maliyet.</t>
+        </is>
+      </c>
+      <c r="F15" s="17" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr"/>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Gün</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Hazır adım (bittiysen Evet)</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Evet / Hayır</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Not</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="B18" s="38" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" s="39" t="inlineStr">
+        <is>
+          <t>Bütçe alt–üst + 2. el/yeni + 3 model yazıldı</t>
+        </is>
+      </c>
+      <c r="D18" s="15" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="E18" s="15" t="inlineStr">
+        <is>
+          <t>Bütçe aralığı yazıldı, 3 aday seçildi.</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="n"/>
+    </row>
+    <row r="19" ht="28" customHeight="1">
+      <c r="B19" s="38" t="n">
+        <v>2</v>
+      </c>
+      <c r="C19" s="39" t="inlineStr">
+        <is>
+          <t>Ehliyet kontrol + kasko/trafik kaba fiyat + biriktirme yeri</t>
+        </is>
+      </c>
+      <c r="D19" s="15" t="n"/>
+      <c r="E19" s="15" t="n"/>
+      <c r="F19" s="8" t="n"/>
+    </row>
+    <row r="20" ht="28" customHeight="1">
+      <c r="B20" s="38" t="n">
+        <v>3</v>
+      </c>
+      <c r="C20" s="39" t="inlineStr">
+        <is>
+          <t>5 ilan kaydedildi, 2 satıcıya mesaj</t>
+        </is>
+      </c>
+      <c r="D20" s="15" t="n"/>
+      <c r="E20" s="15" t="n"/>
+      <c r="F20" s="8" t="n"/>
+    </row>
+    <row r="21" ht="28" customHeight="1">
+      <c r="B21" s="38" t="n">
+        <v>4</v>
+      </c>
+      <c r="C21" s="39" t="inlineStr">
+        <is>
+          <t>İlk küçük transfer yapıldı</t>
+        </is>
+      </c>
+      <c r="D21" s="15" t="n"/>
+      <c r="E21" s="15" t="n"/>
+      <c r="F21" s="8" t="n"/>
+    </row>
+    <row r="22" ht="28" customHeight="1">
+      <c r="B22" s="38" t="n">
+        <v>5</v>
+      </c>
+      <c r="C22" s="39" t="inlineStr">
+        <is>
+          <t>Galeride / park yerinde ‘sürücü’ günü</t>
+        </is>
+      </c>
+      <c r="D22" s="15" t="n"/>
+      <c r="E22" s="15" t="n"/>
+      <c r="F22" s="8" t="n"/>
+    </row>
+    <row r="23" ht="28" customHeight="1">
+      <c r="B23" s="38" t="n">
+        <v>6</v>
+      </c>
+      <c r="C23" s="39" t="inlineStr">
+        <is>
+          <t>1 fiyat veya ekspertiz soruldu</t>
+        </is>
+      </c>
+      <c r="D23" s="15" t="n"/>
+      <c r="E23" s="15" t="n"/>
+      <c r="F23" s="8" t="n"/>
+    </row>
+    <row r="24" ht="28" customHeight="1">
+      <c r="B24" s="38" t="n">
+        <v>7</v>
+      </c>
+      <c r="C24" s="39" t="inlineStr">
+        <is>
+          <t>Adaylar 1–2’ye indi, 21 günlük kilit yazıldı</t>
+        </is>
+      </c>
+      <c r="D24" s="15" t="n"/>
+      <c r="E24" s="15" t="n"/>
+      <c r="F24" s="8" t="n"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="18">
+        <f>IF(COUNTIF(D18:D24,"Evet")=7,"7 araba adımı tamam. 21 güne uzat.","Kalan adım: "&amp;(7-COUNTIF(D18:D24,"Evet"))&amp;" — teknik ekleme, eksik günü bitir.")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="30">
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="B26:F26"/>
+    <mergeCell ref="E21:F21"/>
+  </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="C6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"2. el,Yeni,Kararsız"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D18 D19 D20 D21 D22 D23 D24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Evet,Hayır"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="00C99A4A"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:E14"/>
+  <dimension ref="A2:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1911,222 +2305,266 @@
       </c>
     </row>
     <row r="5" ht="32" customHeight="1">
-      <c r="B5" s="35" t="inlineStr">
+      <c r="B5" s="40" t="inlineStr">
         <is>
           <t>Bu hafta</t>
         </is>
       </c>
-      <c r="C5" s="36" t="inlineStr">
+      <c r="C5" s="41" t="inlineStr">
         <is>
           <t>Neville Goddard — Feeling is the Secret</t>
         </is>
       </c>
-      <c r="D5" s="36" t="inlineStr">
+      <c r="D5" s="41" t="inlineStr">
         <is>
           <t>SATS, uykunun eşiği, his</t>
         </is>
       </c>
-      <c r="E5" s="37" t="inlineStr">
+      <c r="E5" s="42" t="inlineStr">
         <is>
           <t>Kısa. Önce bunu bitir.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1">
-      <c r="B6" s="35" t="inlineStr">
+      <c r="B6" s="40" t="inlineStr">
         <is>
           <t>Bu hafta</t>
         </is>
       </c>
-      <c r="C6" s="38" t="inlineStr">
+      <c r="C6" s="43" t="inlineStr">
         <is>
           <t>Neville Goddard — The Power of Awareness</t>
         </is>
       </c>
-      <c r="D6" s="38" t="inlineStr">
+      <c r="D6" s="43" t="inlineStr">
         <is>
           <t>Kimlik / varsayım / sonda yaşamak</t>
         </is>
       </c>
-      <c r="E6" s="39" t="inlineStr">
+      <c r="E6" s="44" t="inlineStr">
         <is>
           <t>Cümleyi kimlik haline getirir.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1">
-      <c r="B7" s="35" t="inlineStr">
+      <c r="B7" s="40" t="inlineStr">
         <is>
           <t>Bu hafta</t>
         </is>
       </c>
-      <c r="C7" s="36" t="inlineStr">
+      <c r="C7" s="41" t="inlineStr">
         <is>
           <t>woopmylife.org</t>
         </is>
       </c>
-      <c r="D7" s="36" t="inlineStr">
+      <c r="D7" s="41" t="inlineStr">
         <is>
           <t>Wish-Outcome-Obstacle-Plan</t>
         </is>
       </c>
-      <c r="E7" s="37" t="inlineStr">
+      <c r="E7" s="42" t="inlineStr">
         <is>
           <t>5 dakikalık resmi araç.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1">
-      <c r="B8" s="35" t="inlineStr">
+      <c r="B8" s="40" t="inlineStr">
         <is>
           <t>Bu hafta</t>
         </is>
       </c>
-      <c r="C8" s="38" t="inlineStr">
+      <c r="C8" s="43" t="inlineStr">
         <is>
           <t>Gollwitzer — implementation intentions</t>
         </is>
       </c>
-      <c r="D8" s="38" t="inlineStr">
+      <c r="D8" s="43" t="inlineStr">
         <is>
           <t>Eğer-o zaman planlarının etkisi</t>
         </is>
       </c>
-      <c r="E8" s="39" t="inlineStr">
+      <c r="E8" s="44" t="inlineStr">
         <is>
           <t>d ≈ 0.65; niyeti eyleme bağlar.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1">
-      <c r="B9" s="40" t="inlineStr">
+      <c r="B9" s="45" t="inlineStr">
         <is>
           <t>Sonra</t>
         </is>
       </c>
-      <c r="C9" s="36" t="inlineStr">
+      <c r="C9" s="41" t="inlineStr">
         <is>
           <t>Gabriele Oettingen — Rethinking Positive Thinking</t>
         </is>
       </c>
-      <c r="D9" s="36" t="inlineStr">
+      <c r="D9" s="41" t="inlineStr">
         <is>
           <t>Neden sadece hayal yetmez</t>
         </is>
       </c>
-      <c r="E9" s="37" t="inlineStr">
+      <c r="E9" s="42" t="inlineStr">
         <is>
           <t>WOOP’un kitabı.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1">
-      <c r="B10" s="40" t="inlineStr">
+      <c r="B10" s="45" t="inlineStr">
         <is>
           <t>Sonra</t>
         </is>
       </c>
-      <c r="C10" s="38" t="inlineStr">
+      <c r="C10" s="43" t="inlineStr">
         <is>
           <t>Neville — The Law and the Promise</t>
         </is>
       </c>
-      <c r="D10" s="38" t="inlineStr">
+      <c r="D10" s="43" t="inlineStr">
         <is>
           <t>Uygulama hikâyeleri</t>
         </is>
       </c>
-      <c r="E10" s="39" t="inlineStr">
+      <c r="E10" s="44" t="inlineStr">
         <is>
           <t>Teknik oturduktan sonra.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1">
-      <c r="B11" s="40" t="inlineStr">
+      <c r="B11" s="45" t="inlineStr">
         <is>
           <t>Sonra</t>
         </is>
       </c>
-      <c r="C11" s="36" t="inlineStr">
+      <c r="C11" s="41" t="inlineStr">
         <is>
           <t>James Clear — Atomic Habits</t>
         </is>
       </c>
-      <c r="D11" s="36" t="inlineStr">
+      <c r="D11" s="41" t="inlineStr">
         <is>
           <t>Küçük günlük adım</t>
         </is>
       </c>
-      <c r="E11" s="37" t="inlineStr">
+      <c r="E11" s="42" t="inlineStr">
         <is>
           <t>WOOP’un davranış yüzü.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1">
-      <c r="B12" s="41" t="inlineStr">
+      <c r="B12" s="40" t="inlineStr">
+        <is>
+          <t>Bu hafta</t>
+        </is>
+      </c>
+      <c r="C12" s="43" t="inlineStr">
+        <is>
+          <t>Sahibinden / yetkili galeri</t>
+        </is>
+      </c>
+      <c r="D12" s="43" t="inlineStr">
+        <is>
+          <t>3 aday, gerçek fiyat</t>
+        </is>
+      </c>
+      <c r="E12" s="44" t="inlineStr">
+        <is>
+          <t>Saatlerce bakma; 2 mesaj at.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="B13" s="40" t="inlineStr">
+        <is>
+          <t>Bu hafta</t>
+        </is>
+      </c>
+      <c r="C13" s="41" t="inlineStr">
+        <is>
+          <t>Trafik sigortası + kasko teklifi</t>
+        </is>
+      </c>
+      <c r="D13" s="41" t="inlineStr">
+        <is>
+          <t>Aylık gerçek maliyet</t>
+        </is>
+      </c>
+      <c r="E13" s="42" t="inlineStr">
+        <is>
+          <t>Araba fiyatının yanında bunu da yaz.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="32" customHeight="1">
+      <c r="B14" s="46" t="inlineStr">
         <is>
           <t>Uzak dur</t>
         </is>
       </c>
-      <c r="C12" s="38" t="inlineStr">
-        <is>
-          <t>Sonsuz koç reeli / anında zengin ol vaadi</t>
-        </is>
-      </c>
-      <c r="D12" s="38" t="inlineStr">
+      <c r="C14" s="43" t="inlineStr">
+        <is>
+          <t>“Evren bugün araba yollar” reelleri</t>
+        </is>
+      </c>
+      <c r="D14" s="43" t="inlineStr">
         <is>
           <t>Dağıtır</t>
         </is>
       </c>
-      <c r="E12" s="39" t="inlineStr">
+      <c r="E14" s="44" t="inlineStr">
         <is>
           <t>7 gün protokolü bozar.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="32" customHeight="1">
-      <c r="B13" s="41" t="inlineStr">
+    <row r="15" ht="32" customHeight="1">
+      <c r="B15" s="46" t="inlineStr">
         <is>
           <t>Uzak dur</t>
         </is>
       </c>
-      <c r="C13" s="36" t="inlineStr">
-        <is>
-          <t>Başkasının iradesini manipüle etme teknikleri</t>
-        </is>
-      </c>
-      <c r="D13" s="36" t="inlineStr">
-        <is>
-          <t>Zararlı ve boşa</t>
-        </is>
-      </c>
-      <c r="E13" s="37" t="inlineStr">
-        <is>
-          <t>Karşılıklı, serbest hali iste.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="32" customHeight="1">
-      <c r="B14" s="41" t="inlineStr">
+      <c r="C15" s="41" t="inlineStr">
+        <is>
+          <t>10 modeli aynı anda hayal</t>
+        </is>
+      </c>
+      <c r="D15" s="41" t="inlineStr">
+        <is>
+          <t>Odak kaçması</t>
+        </is>
+      </c>
+      <c r="E15" s="42" t="inlineStr">
+        <is>
+          <t>En fazla 3 aday.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="32" customHeight="1">
+      <c r="B16" s="46" t="inlineStr">
         <is>
           <t>Uzak dur</t>
         </is>
       </c>
-      <c r="C14" s="38" t="inlineStr">
-        <is>
-          <t>Aynı anda 10 yöntem</t>
-        </is>
-      </c>
-      <c r="D14" s="38" t="inlineStr">
-        <is>
-          <t>Odak kaçması</t>
-        </is>
-      </c>
-      <c r="E14" s="39" t="inlineStr">
-        <is>
-          <t>Tek protokol, 7 gün.</t>
+      <c r="C16" s="43" t="inlineStr">
+        <is>
+          <t>Birinin sana almasını beklemek</t>
+        </is>
+      </c>
+      <c r="D16" s="43" t="inlineStr">
+        <is>
+          <t>Pasiflik</t>
+        </is>
+      </c>
+      <c r="E16" s="44" t="inlineStr">
+        <is>
+          <t>Biriktir / kredi / 2. el senin adımın.</t>
         </is>
       </c>
     </row>

</xml_diff>